<commit_message>
Add fault-tolerant enhancements to IT ticketing workflow. Update main workflow to include AI summarization, processing stages, and improved error handling. Revise workflow guide for clarity and detail. Update Excel workbook structure to support new features.
</commit_message>
<xml_diff>
--- a/assets/IT Support Tickets NGI.xlsx
+++ b/assets/IT Support Tickets NGI.xlsx
@@ -21,12 +21,15 @@
     <definedName name="SLA_Low">Configuration!$B$10</definedName>
     <definedName name="List_Categories">'Categories'!$A$2:$A$9</definedName>
     <definedName name="List_Engineers">'Users'!$A$2:$A$5</definedName>
-    <definedName name="List_Status">'Users'!$F$2:$F$6</definedName>
+    <definedName name="List_Status">'Users'!$F$2:$F$7</definedName>
     <definedName name="List_Priority">'Users'!$G$2:$G$4</definedName>
     <definedName name="List_Department">'Users'!$H$2:$H$9</definedName>
     <definedName name="List_Escalation">'Users'!$I$2:$I$5</definedName>
     <definedName name="List_Resolution">'Users'!$J$2:$J$10</definedName>
     <definedName name="List_ClosureReason">'Users'!$K$2:$K$7</definedName>
+    <definedName name="List_ProcessingStage">'Users'!$L$2:$L$5</definedName>
+    <definedName name="List_AckSent">'Users'!$M$2:$M$3</definedName>
+    <definedName name="List_AIPriority">'Users'!$N$2:$N$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -131,12 +134,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -150,6 +149,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FECACA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FDE68A"/>
         </patternFill>
       </fill>
     </dxf>
@@ -178,13 +184,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FCA5A5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FDE68A"/>
         </patternFill>
       </fill>
     </dxf>
@@ -304,12 +303,12 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Dashboard'!$D$4:$D$8</f>
+              <f>'Dashboard'!$D$4:$D$9</f>
             </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$4:$E$8</f>
+              <f>'Dashboard'!$E$4:$E$9</f>
             </numRef>
           </val>
         </ser>
@@ -413,7 +412,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2880000"/>
@@ -435,7 +434,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>13</row>
+      <row>14</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4320000" cy="2880000"/>
@@ -457,9 +456,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ITTickets" displayName="ITTickets" ref="A1:AA4" headerRowCount="1">
-  <autoFilter ref="A1:AA4"/>
-  <tableColumns count="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ITTickets" displayName="ITTickets" ref="A1:AF4" headerRowCount="1">
+  <autoFilter ref="A1:AF4"/>
+  <tableColumns count="32">
     <tableColumn id="1" name="Ticket ID"/>
     <tableColumn id="2" name="Created Date"/>
     <tableColumn id="3" name="Created Time"/>
@@ -485,8 +484,13 @@
     <tableColumn id="23" name="Escalation Level"/>
     <tableColumn id="24" name="Resolution"/>
     <tableColumn id="25" name="Closure Reason"/>
-    <tableColumn id="26" name="Ticket Age Days"/>
-    <tableColumn id="27" name="SLA Remaining Hours"/>
+    <tableColumn id="26" name="Processing Stage"/>
+    <tableColumn id="27" name="Ack Sent"/>
+    <tableColumn id="28" name="AI Issue Summary"/>
+    <tableColumn id="29" name="AI Priority"/>
+    <tableColumn id="30" name="AI Scope"/>
+    <tableColumn id="31" name="Ticket Age Days"/>
+    <tableColumn id="32" name="SLA Remaining Hours"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -796,7 +800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -959,57 +963,76 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Tickets!$L$2:$L$5000,"Closed")</f>
+        <f>COUNTIF(Tickets!$L$2:$L$5000,"Needs Review")</f>
         <v/>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Needs Review</t>
         </is>
       </c>
       <c r="E8" s="4">
-        <f>COUNTIF(Tickets!$L$2:$L$5000,"Closed")</f>
+        <f>COUNTIF(Tickets!$L$2:$L$5000,"Needs Review")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>High Priority Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIFS(Tickets!$I$2:$I$5000,"High",Tickets!$L$2:$L$5000,"&lt;&gt;Closed")</f>
+        <f>COUNTIF(Tickets!$L$2:$L$5000,"Closed")</f>
+        <v/>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="E9" s="4">
+        <f>COUNTIF(Tickets!$L$2:$L$5000,"Closed")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Unassigned</t>
+          <t>High Priority Open</t>
         </is>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Tickets!$M$2:$M$5000,"Unassigned")</f>
+        <f>COUNTIFS(Tickets!$I$2:$I$5000,"High",Tickets!$L$2:$L$5000,"&lt;&gt;Closed")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>COUNTIF(Tickets!$M$2:$M$5000,"Unassigned")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>Avg Age (Open Days)</t>
         </is>
       </c>
-      <c r="B11" s="5">
-        <f>IFERROR(AVERAGEIF(Tickets!$L$2:$L$5000,"&lt;&gt;Closed",Tickets!$Z$2:$Z$5000),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12"/>
+      <c r="B12" s="5">
+        <f>IFERROR(AVERAGEIF(Tickets!$L$2:$L$5000,"&lt;&gt;Closed",Tickets!$AE$2:$AE$5000),0)</f>
+        <v/>
+      </c>
+    </row>
     <row r="13"/>
     <row r="14"/>
     <row r="15"/>
@@ -1021,40 +1044,30 @@
     <row r="21"/>
     <row r="22"/>
     <row r="23"/>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>Engineer Workload (non-closed)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Open Tickets</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Unassigned</t>
-        </is>
-      </c>
-      <c r="B26" s="4">
-        <f>COUNTIFS(Tickets!$M$2:$M$5000,A26,Tickets!$L$2:$L$5000,"&lt;&gt;Closed")</f>
-        <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Rushak Pachpande</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="B27" s="4">
@@ -1065,7 +1078,7 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>IT Engineer 1</t>
+          <t>Rushak Pachpande</t>
         </is>
       </c>
       <c r="B28" s="4">
@@ -1076,11 +1089,22 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>IT Engineer 2</t>
+          <t>IT Engineer 1</t>
         </is>
       </c>
       <c r="B29" s="4">
         <f>COUNTIFS(Tickets!$M$2:$M$5000,A29,Tickets!$L$2:$L$5000,"&lt;&gt;Closed")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>IT Engineer 2</t>
+        </is>
+      </c>
+      <c r="B30" s="4">
+        <f>COUNTIFS(Tickets!$M$2:$M$5000,A30,Tickets!$L$2:$L$5000,"&lt;&gt;Closed")</f>
         <v/>
       </c>
     </row>
@@ -1099,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA4"/>
+  <dimension ref="A1:AF4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1119,7 +1143,7 @@
     <col width="35" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
     <col width="21" customWidth="1" min="19" max="19"/>
     <col width="21" customWidth="1" min="20" max="20"/>
     <col width="28" customWidth="1" min="21" max="21"/>
@@ -1127,8 +1151,13 @@
     <col width="18" customWidth="1" min="23" max="23"/>
     <col width="19" customWidth="1" min="24" max="24"/>
     <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="42" customWidth="1" min="26" max="26"/>
-    <col width="42" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="40" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="28" customWidth="1" min="30" max="30"/>
+    <col width="42" customWidth="1" min="31" max="31"/>
+    <col width="42" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1259,10 +1288,35 @@
       </c>
       <c r="Z1" s="2" t="inlineStr">
         <is>
+          <t>Processing Stage</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>Ack Sent</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>AI Issue Summary</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>AI Priority</t>
+        </is>
+      </c>
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>AI Scope</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
           <t>Ticket Age Days</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>SLA Remaining Hours</t>
         </is>
@@ -1275,7 +1329,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
@@ -1350,11 +1404,11 @@
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>Processed/Open Tickets</t>
+          <t>Open Tickets</t>
         </is>
       </c>
       <c r="S2" s="8" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="T2" s="7" t="n"/>
       <c r="U2" s="9" t="inlineStr"/>
@@ -1370,12 +1424,37 @@
       </c>
       <c r="X2" s="7" t="inlineStr"/>
       <c r="Y2" s="7" t="inlineStr"/>
-      <c r="Z2" s="10">
+      <c r="Z2" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="AA2" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB2" s="9" t="inlineStr">
+        <is>
+          <t>VPN connection fails with error 809 after a Windows update.</t>
+        </is>
+      </c>
+      <c r="AC2" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="AD2" s="9" t="inlineStr">
+        <is>
+          <t>VPN client / Engineering user Priya Sharma</t>
+        </is>
+      </c>
+      <c r="AE2" s="10">
         <f>IF(A2="","",IF(L2="Closed",IF(T2="",0,MAX(0,T2-B2)),MAX(0,TODAY()-B2)))</f>
         <v/>
       </c>
-      <c r="AA2" s="11">
-        <f>IF(OR(A2="",L2="Closed"),"",IF(I2="High",SLA_High,IF(I2="Low",SLA_Low,SLA_Medium))-Z2*24)</f>
+      <c r="AF2" s="11">
+        <f>IF(OR(A2="",L2="Closed"),"",IF(I2="High",SLA_High,IF(I2="Low",SLA_Low,SLA_Medium))-AE2*24)</f>
         <v/>
       </c>
     </row>
@@ -1386,7 +1465,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>46231</v>
+        <v>46232</v>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
@@ -1457,11 +1536,11 @@
       </c>
       <c r="R3" s="7" t="inlineStr">
         <is>
-          <t>Processed/Open Tickets</t>
+          <t>Open Tickets</t>
         </is>
       </c>
       <c r="S3" s="8" t="n">
-        <v>46234</v>
+        <v>46235</v>
       </c>
       <c r="T3" s="7" t="n"/>
       <c r="U3" s="9" t="inlineStr"/>
@@ -1477,12 +1556,37 @@
       </c>
       <c r="X3" s="7" t="inlineStr"/>
       <c r="Y3" s="7" t="inlineStr"/>
-      <c r="Z3" s="10">
+      <c r="Z3" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="AA3" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB3" s="9" t="inlineStr">
+        <is>
+          <t>Outlook search returns no results for recent mail.</t>
+        </is>
+      </c>
+      <c r="AC3" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="AD3" s="9" t="inlineStr">
+        <is>
+          <t>Outlook / Sales user Amit Patel</t>
+        </is>
+      </c>
+      <c r="AE3" s="10">
         <f>IF(A3="","",IF(L3="Closed",IF(T3="",0,MAX(0,T3-B3)),MAX(0,TODAY()-B3)))</f>
         <v/>
       </c>
-      <c r="AA3" s="11">
-        <f>IF(OR(A3="",L3="Closed"),"",IF(I3="High",SLA_High,IF(I3="Low",SLA_Low,SLA_Medium))-Z3*24)</f>
+      <c r="AF3" s="11">
+        <f>IF(OR(A3="",L3="Closed"),"",IF(I3="High",SLA_High,IF(I3="Low",SLA_Low,SLA_Medium))-AE3*24)</f>
         <v/>
       </c>
     </row>
@@ -1493,7 +1597,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>46229</v>
+        <v>46230</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
@@ -1568,14 +1672,14 @@
       </c>
       <c r="R4" s="7" t="inlineStr">
         <is>
-          <t>Processed/Closed</t>
+          <t>Processed</t>
         </is>
       </c>
       <c r="S4" s="8" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="T4" s="8" t="n">
-        <v>46233</v>
+        <v>46234</v>
       </c>
       <c r="U4" s="9" t="inlineStr">
         <is>
@@ -1598,12 +1702,37 @@
           <t>Completed</t>
         </is>
       </c>
-      <c r="Z4" s="10">
+      <c r="Z4" s="7" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="AA4" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="AB4" s="9" t="inlineStr">
+        <is>
+          <t>Request for Windows 11 laptop setup for a new joiner.</t>
+        </is>
+      </c>
+      <c r="AC4" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="AD4" s="9" t="inlineStr">
+        <is>
+          <t>Laptop / HR new joiner</t>
+        </is>
+      </c>
+      <c r="AE4" s="10">
         <f>IF(A4="","",IF(L4="Closed",IF(T4="",0,MAX(0,T4-B4)),MAX(0,TODAY()-B4)))</f>
         <v/>
       </c>
-      <c r="AA4" s="11">
-        <f>IF(OR(A4="",L4="Closed"),"",IF(I4="High",SLA_High,IF(I4="Low",SLA_Low,SLA_Medium))-Z4*24)</f>
+      <c r="AF4" s="11">
+        <f>IF(OR(A4="",L4="Closed"),"",IF(I4="High",SLA_High,IF(I4="Low",SLA_Low,SLA_Medium))-AE4*24)</f>
         <v/>
       </c>
     </row>
@@ -1616,31 +1745,34 @@
       <formula>"New"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="1">
+      <formula>"Needs Review"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
       <formula>"Pending"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:I5000">
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M5000">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="1">
       <formula>"Unassigned"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA2:AA5000">
-    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="6">
+  <conditionalFormatting sqref="AF2:AF5000">
+    <cfRule type="cellIs" priority="9" operator="lessThan" dxfId="6">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="11">
     <dataValidation sqref="I2:I5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
       <formula1>=List_Priority</formula1>
     </dataValidation>
@@ -1665,6 +1797,15 @@
     <dataValidation sqref="Y2:Y5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
       <formula1>=List_ClosureReason</formula1>
     </dataValidation>
+    <dataValidation sqref="Z2:Z5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
+      <formula1>=List_ProcessingStage</formula1>
+    </dataValidation>
+    <dataValidation sqref="AA2:AA5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
+      <formula1>=List_AckSent</formula1>
+    </dataValidation>
+    <dataValidation sqref="AC2:AC5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Please select a value from the dropdown list." type="list">
+      <formula1>=List_AIPriority</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -1814,7 +1955,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1967,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31 17:40:25</t>
+          <t>2026-08-01 01:10:46</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1982,7 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>Upload this workbook to OneDrive/SharePoint under the IT Support account. In n8n Excel nodes, reselect this workbook and the ITTickets / AuditLog tables after upload (workbook and table IDs are tenant-specific). CreatedDate / ClosedDate are real Excel dates (display dd-mm-yyyy).</t>
+          <t>Upload this workbook to OneDrive/SharePoint under the IT Support account. In n8n Excel nodes, reselect this workbook and the ITTickets / AuditLog tables after upload (workbook and table IDs are tenant-specific). CreatedDate / ClosedDate are real Excel dates (display dd-mm-yyyy). Processing Stage / Ack Sent enable fault-tolerant resume; AI columns hold LLM summaries. Outlook folders: Inbox, Open Tickets, Processed.</t>
         </is>
       </c>
     </row>
@@ -1942,7 +2083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1950,12 +2091,15 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="27" customWidth="1" min="10" max="10"/>
     <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2009,6 +2153,21 @@
           <t>ClosureReasonList</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ProcessingStageList</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>AckSentList</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>AIPriorityList</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -2061,6 +2220,21 @@
           <t>Completed</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2113,6 +2287,21 @@
           <t>Cancelled by User</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Acked</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -2165,6 +2354,16 @@
           <t>Duplicate Ticket</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Complete</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -2208,30 +2407,45 @@
           <t>No Response from User</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>NeedsReview</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="F6" t="inlineStr">
         <is>
+          <t>Needs Review</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Resolved - Access Granted</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Out of Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Closed</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Operations</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Resolved - Access Granted</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Out of Scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
       <c r="H7" t="inlineStr">
         <is>
           <t>Marketing</t>
@@ -2336,7 +2550,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31 17:40:25</t>
+          <t>2026-08-01 01:10:46</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">

</xml_diff>